<commit_message>
Enhance EntityExtractor with salary range and reddit company pattern matching
</commit_message>
<xml_diff>
--- a/module_1_scraping_engine/data/output/archetype_d_test_scraped_data.xlsx
+++ b/module_1_scraping_engine/data/output/archetype_d_test_scraped_data.xlsx
@@ -517,7 +517,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>₹40,000</t>
+          <t>₹40,000/mo</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -537,7 +537,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-10-16T15:44:31.132284+00:00</t>
+          <t>2026-10-16T15:48:21.004047+00:00</t>
         </is>
       </c>
     </row>
@@ -599,7 +599,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-10-16T15:44:31.133283+00:00</t>
+          <t>2026-10-16T15:48:21.004047+00:00</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-10-16T15:44:31.133283+00:00</t>
+          <t>2026-10-16T15:48:21.004047+00:00</t>
         </is>
       </c>
     </row>
@@ -723,7 +723,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-10-16T15:44:31.705194+00:00</t>
+          <t>2026-10-16T15:48:21.585402+00:00</t>
         </is>
       </c>
     </row>
@@ -785,7 +785,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-10-16T15:44:32.295492+00:00</t>
+          <t>2026-10-16T15:48:22.345100+00:00</t>
         </is>
       </c>
     </row>
@@ -827,7 +827,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>18 - 25 LPA</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-10-16T15:44:32.296492+00:00</t>
+          <t>2026-10-16T15:48:22.345100+00:00</t>
         </is>
       </c>
     </row>
@@ -889,7 +889,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>$2,500</t>
+          <t>$2,500/mo</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -909,7 +909,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-10-16T15:44:32.296492+00:00</t>
+          <t>2026-10-16T15:48:22.346100+00:00</t>
         </is>
       </c>
     </row>
@@ -931,7 +931,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Developer</t>
+          <t>Supabase</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>$80,000</t>
+          <t>$80,000 - $110,000/yr</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -971,7 +971,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-10-16T15:44:32.297489+00:00</t>
+          <t>2026-10-16T15:48:22.346100+00:00</t>
         </is>
       </c>
     </row>
@@ -993,7 +993,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Direct Tech Hiring</t>
+          <t>Zerodha</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-10-16T15:44:32.297489+00:00</t>
+          <t>2026-10-16T15:48:22.346100+00:00</t>
         </is>
       </c>
     </row>
@@ -1095,7 +1095,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-10-16T15:44:32.297489+00:00</t>
+          <t>2026-10-16T15:48:22.346100+00:00</t>
         </is>
       </c>
     </row>
@@ -1157,7 +1157,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-10-16T15:44:32.298488+00:00</t>
+          <t>2026-10-16T15:48:22.346100+00:00</t>
         </is>
       </c>
     </row>
@@ -1219,7 +1219,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-10-16T15:44:32.298488+00:00</t>
+          <t>2026-10-16T15:48:22.346100+00:00</t>
         </is>
       </c>
     </row>
@@ -1281,7 +1281,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-10-16T15:44:32.298488+00:00</t>
+          <t>2026-10-16T15:48:22.347098+00:00</t>
         </is>
       </c>
     </row>
@@ -1343,7 +1343,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-10-16T15:44:32.298488+00:00</t>
+          <t>2026-10-16T15:48:22.347098+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>